<commit_message>
feat(seo): Phase 0 — CTR + brand schema enrichment (UA/RU/EN homes + pricing)
- RU/EN home: extended LocalBusiness (logo, sameAs, priceRange UAH 18-650,
  areaServed, knowsAbout, aggregateRating) + WebSite schema
- EN home title: $0.40 -> EUR 0.40/order (EU market relevance)
- EN /prices: LocalBusiness schema extended to match UA/RU quality
- Fixed broken /images/mtp-logo.webp (copied from Tilda legacy)
- Added semantic core dynamic tracking: JSON-backed progress log +
  10-sheet Excel with Completion log tab, DONE markers, color coding
- Re-run scripts/gen-semantic-excel.py after updating progress JSON

Co-Authored-By: claude-flow <ruv@ruv.net>
</commit_message>
<xml_diff>
--- a/docs/SEMANTIC_CORE_ROADMAP.xlsx
+++ b/docs/SEMANTIC_CORE_ROADMAP.xlsx
@@ -16,15 +16,17 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🔄 v1 vs v2" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🏢 Competitors" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🔍 Top queries" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📅 Completion log" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'✅ Current inventory'!$A$1:$J$179</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'🎯 Striking distance'!$A$1:$M$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'⚠️ Gap analysis'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'🗓️ Roadmap Phases'!$A$1:$G$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'🗓️ Roadmap Phases'!$A$1:$J$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'🔄 v1 vs v2'!$A$1:$D$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'🏢 Competitors'!$A$1:$F$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'🔍 Top queries'!$A$1:$G$335</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'📅 Completion log'!$A$3:$F$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -33,7 +35,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -60,6 +62,10 @@
       <b val="1"/>
       <color rgb="00E63329"/>
       <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001B5E20"/>
     </font>
     <font>
       <b val="1"/>
@@ -122,7 +128,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -152,7 +158,8 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -910,6 +917,317 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="80" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>COMPLETION LOG — хронологія виконаних задач</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C3" s="12" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="D3" s="12" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="E3" s="12" t="inlineStr">
+        <is>
+          <t>Phase</t>
+        </is>
+      </c>
+      <c r="F3" s="12" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Переписати home title + meta з ціною</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>✅ DONE</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>pending-phase0</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Phase 0</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>UA home вже мав 'від 18 грн' в title/desc. RU home extended LocalBusiness schema (logo, sameAs, priceRange, areaServed, knowsAbout) + WebSite schema. EN home title changed from '$0.40' to '€0.40/order</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Organization schema для brand search</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>✅ DONE</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>pending-phase0</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Phase 0</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>UA home had full LocalBusiness schema already. Extended RU + EN home with: logo, image, sameAs (FB/LinkedIn/Telegram), priceRange 'UAH 18 - UAH 650', aggregateRating, areaServed, knowsAbout. Fixed bro</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Оновити /tsiny/ /tsenu/ /prices/ meta</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>✅ PARTIAL</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>pending-phase0</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Phase 0</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>UA /tsiny/ and RU /tsenu/ already had '18 грн' in title/desc/FAQ schema — no change needed. EN /prices/ extended LocalBusiness schema with logo, sameAs, priceRange to match UA/RU quality.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Видалити дубль generate_lead/form_submit на EN thanks</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>✅ DONE</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>ff0bfe9</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Fix A. en/thanks.astro: removed form_submit + generate_lead + dataLayer.push; kept only AdWords conversion event. Eliminates GA4 lead double-count for EN traffic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Видалити дубль GTM noscript iframe з 23 blog pages</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>✅ DONE</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>8a744c5</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Fix B. Removed duplicate noscript iframe from 23 files; Base.astro:172 retained as single source of truth. 1 line deleted per file, no other changes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Tilda 301 clean sweep (59 legacy URLs)</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>✅ DONE</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>prior-session</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>vercel.json — 5 specific Tier 1 redirects + 3 catch-all patterns for /blog/tpost/, /ua/blog/tpost/, /en/blog/tpost/. All point directly to /ua/blog/ or /ua/about/ (no chained redirects). 132 redirects</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>GSC full audit + competitor research</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>✅ DONE</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>ff0bfe9</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Analysis</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Generated docs/gsc/full-pages.{csv,json}, full-queries.{csv,json}, opportunities.{csv,json}, competitor-gap-research.md. 178 pages, 334 queries, 29 clicks, 4329 impressions (90d baseline).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Claim Google Business Profile</t>
+        </is>
+      </c>
+      <c r="C11" s="14" t="inlineStr">
+        <is>
+          <t>✅ MANUAL_USER_ACTION</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Phase 0</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>External task — user must claim at business.google.com. Recommended: entity name 'MTP Group Fulfillment', category 'Logistics service', both addresses (Щасливе + Білогородка), phone +380501444645, hou</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A3:F11"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -10371,7 +10689,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:J39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10379,8 +10697,11 @@
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
     <col width="35" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -10419,6 +10740,21 @@
           <t>Expected impact</t>
         </is>
       </c>
+      <c r="H1" s="12" t="inlineStr">
+        <is>
+          <t>Done date</t>
+        </is>
+      </c>
+      <c r="I1" s="12" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="J1" s="12" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
@@ -10446,14 +10782,29 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="F2" s="15" t="inlineStr">
+        <is>
+          <t>✅ DONE</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
           <t>+40-60 clicks/mo</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>pending-phase0</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>UA home вже мав 'від 18 грн' в title/desc. RU home extended LocalBusiness schema (logo, sameAs, priceRange, areaServed, knowsAbout) + WebSite schema. EN home title changed from '$0.40' to '€0.40/order' (EU-relevant); LocalBusiness extended. Real 'price in meta' was already present — actual fix was schema enrichment for brand signals.</t>
         </is>
       </c>
     </row>
@@ -10483,14 +10834,29 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="F3" s="15" t="inlineStr">
+        <is>
+          <t>✅ DONE</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
           <t>+20-40 clicks/mo</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>pending-phase0</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>UA home had full LocalBusiness schema already. Extended RU + EN home with: logo, image, sameAs (FB/LinkedIn/Telegram), priceRange 'UAH 18 - UAH 650', aggregateRating, areaServed, knowsAbout. Fixed broken /images/mtp-logo.webp reference (was missing, copied from Tilda legacy filename).</t>
         </is>
       </c>
     </row>
@@ -10520,14 +10886,29 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="F4" s="15" t="inlineStr">
+        <is>
+          <t>✅ PARTIAL</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
           <t>+15-25 clicks/mo</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>pending-phase0</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>UA /tsiny/ and RU /tsenu/ already had '18 грн' in title/desc/FAQ schema — no change needed. EN /prices/ extended LocalBusiness schema with logo, sameAs, priceRange to match UA/RU quality.</t>
         </is>
       </c>
     </row>
@@ -10557,14 +10938,19 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="F5" s="14" t="inlineStr">
+        <is>
+          <t>✅ MANUAL_USER_ACTION</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
           <t>Brand CTR</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>External task — user must claim at business.google.com. Recommended: entity name 'MTP Group Fulfillment', category 'Logistics service', both addresses (Щасливе + Білогородка), phone +380501444645, hours Mo-Su 08:00-20:00.</t>
         </is>
       </c>
     </row>
@@ -10604,6 +10990,9 @@
           <t>+100-200 clicks/mo через 2-3 міс</t>
         </is>
       </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
@@ -10641,6 +11030,9 @@
           <t>+40-80 clicks/mo</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -10678,6 +11070,9 @@
           <t>+20-40 clicks/mo</t>
         </is>
       </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
@@ -10715,6 +11110,9 @@
           <t>+30-50 clicks/mo</t>
         </is>
       </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
@@ -10752,6 +11150,9 @@
           <t>+25-40 clicks/mo</t>
         </is>
       </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
@@ -10789,6 +11190,9 @@
           <t>pos 7.3 → 3</t>
         </is>
       </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
@@ -10826,6 +11230,9 @@
           <t>+15-25 clicks/mo</t>
         </is>
       </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="13" t="inlineStr">
@@ -10863,6 +11270,9 @@
           <t>+10-20 clicks/mo</t>
         </is>
       </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="13" t="inlineStr">
@@ -10900,6 +11310,9 @@
           <t>+15-25 clicks/mo</t>
         </is>
       </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="13" t="inlineStr">
@@ -10937,6 +11350,9 @@
           <t>+10-20 clicks/mo</t>
         </is>
       </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="13" t="inlineStr">
@@ -10974,6 +11390,9 @@
           <t>Infrastructure only</t>
         </is>
       </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="13" t="inlineStr">
@@ -11011,6 +11430,9 @@
           <t>+30-50 clicks/mo</t>
         </is>
       </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="13" t="inlineStr">
@@ -11048,6 +11470,9 @@
           <t>+20-30 clicks/mo</t>
         </is>
       </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="13" t="inlineStr">
@@ -11085,6 +11510,9 @@
           <t>+15-25 clicks/mo</t>
         </is>
       </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="13" t="inlineStr">
@@ -11122,6 +11550,9 @@
           <t>+20-40 clicks/mo</t>
         </is>
       </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="13" t="inlineStr">
@@ -11159,6 +11590,9 @@
           <t>+15-30 clicks/mo</t>
         </is>
       </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="13" t="inlineStr">
@@ -11196,6 +11630,9 @@
           <t>+10-20 clicks/mo</t>
         </is>
       </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="13" t="inlineStr">
@@ -11233,6 +11670,9 @@
           <t>+15-25 clicks/mo</t>
         </is>
       </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="13" t="inlineStr">
@@ -11270,6 +11710,9 @@
           <t>+30-50 clicks/mo</t>
         </is>
       </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="13" t="inlineStr">
@@ -11307,6 +11750,9 @@
           <t>+25-40 clicks/mo</t>
         </is>
       </c>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="13" t="inlineStr">
@@ -11344,6 +11790,9 @@
           <t>+20-35 clicks/mo</t>
         </is>
       </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="13" t="inlineStr">
@@ -11381,6 +11830,9 @@
           <t>+15-25 clicks/mo</t>
         </is>
       </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="13" t="inlineStr">
@@ -11418,6 +11870,9 @@
           <t>+15-25 clicks/mo</t>
         </is>
       </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="13" t="inlineStr">
@@ -11455,6 +11910,9 @@
           <t>+10-20 clicks/mo</t>
         </is>
       </c>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="13" t="inlineStr">
@@ -11492,6 +11950,9 @@
           <t>+10-20 clicks/mo</t>
         </is>
       </c>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="13" t="inlineStr">
@@ -11529,6 +11990,9 @@
           <t>+10-20 clicks/mo</t>
         </is>
       </c>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="13" t="inlineStr">
@@ -11566,6 +12030,9 @@
           <t>+30-60 clicks/mo</t>
         </is>
       </c>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="13" t="inlineStr">
@@ -11603,6 +12070,9 @@
           <t>+40-80 clicks/mo</t>
         </is>
       </c>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="13" t="inlineStr">
@@ -11640,6 +12110,9 @@
           <t>+10-20 clicks/mo</t>
         </is>
       </c>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="14" t="inlineStr">
@@ -11677,6 +12150,9 @@
           <t>topic authority</t>
         </is>
       </c>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="14" t="inlineStr">
@@ -11714,6 +12190,9 @@
           <t>+10-20 clicks/mo each</t>
         </is>
       </c>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="14" t="inlineStr">
@@ -11751,6 +12230,9 @@
           <t>Paid+organic sync</t>
         </is>
       </c>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
@@ -11788,6 +12270,9 @@
           <t>Maintenance</t>
         </is>
       </c>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="14" t="inlineStr">
@@ -11825,9 +12310,12 @@
           <t>Consolidate signal</t>
         </is>
       </c>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G39"/>
+  <autoFilter ref="A1:J39"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -12823,7 +13311,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="15" t="inlineStr"/>
+      <c r="A17" s="16" t="inlineStr"/>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
@@ -12831,7 +13319,7 @@
       <c r="F17" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="15" t="inlineStr">
+      <c r="A18" s="16" t="inlineStr">
         <is>
           <t>BOTTOM LINE</t>
         </is>
@@ -12843,7 +13331,7 @@
       <c r="F18" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="15" t="inlineStr">
+      <c r="A19" s="16" t="inlineStr">
         <is>
           <t>MTP не в топ-10 за "фулфілмент для інтернет-магазину"</t>
         </is>
@@ -12859,7 +13347,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="15" t="inlineStr">
+      <c r="A20" s="16" t="inlineStr">
         <is>
           <t>3 pillar gaps MTP:</t>
         </is>
@@ -12871,7 +13359,7 @@
       <c r="F20" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="15" t="inlineStr">
+      <c r="A21" s="16" t="inlineStr">
         <is>
           <t>A: educational "що таке фулфілмент" — 1-2K/mo</t>
         </is>
@@ -12887,7 +13375,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="15" t="inlineStr">
+      <c r="A22" s="16" t="inlineStr">
         <is>
           <t>B: "ТОП операторів" comparison listicles</t>
         </is>
@@ -12903,7 +13391,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="15" t="inlineStr">
+      <c r="A23" s="16" t="inlineStr">
         <is>
           <t>C: marketplace integrations (Rozetka/Prom/OLX)</t>
         </is>
@@ -12919,7 +13407,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="15" t="inlineStr"/>
+      <c r="A24" s="16" t="inlineStr"/>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr"/>
@@ -12927,7 +13415,7 @@
       <c r="F24" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="15" t="inlineStr">
+      <c r="A25" s="16" t="inlineStr">
         <is>
           <t>TOTAL GAP: ~5,000-8,000 monthly UA queries де MTP не в топ-10</t>
         </is>

</xml_diff>

<commit_message>
docs(seo): update progress log with Phase 0 commit SHA (6058d76)
Regenerates SEMANTIC_CORE_ROADMAP.xlsx — Completion log now shows
actual commit for Phase 0 tasks (home title, Organization schema,
pricing meta).

Co-Authored-By: claude-flow <ruv@ruv.net>
</commit_message>
<xml_diff>
--- a/docs/SEMANTIC_CORE_ROADMAP.xlsx
+++ b/docs/SEMANTIC_CORE_ROADMAP.xlsx
@@ -991,7 +991,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>pending-phase0</t>
+          <t>6058d76</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -1023,7 +1023,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>pending-phase0</t>
+          <t>6058d76</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>pending-phase0</t>
+          <t>6058d76</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -10799,7 +10799,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>pending-phase0</t>
+          <t>6058d76</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -10851,7 +10851,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>pending-phase0</t>
+          <t>6058d76</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -10903,7 +10903,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>pending-phase0</t>
+          <t>6058d76</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">

</xml_diff>

<commit_message>
feat(gbp): add Playwright toolkit + optimization plan for 2 verified branches
- scripts/gbp-auth.py: one-time login, saves session to scripts/gbp-session/
- scripts/gbp-audit.py: scrapes both branches (MTPFUL1, MTPFUL2) via SERP admin overlay
- scripts/gbp-edit-scrape.py: edit-panel capture attempt (partial — SERP selectors ambiguous)
- docs/gbp/optimization-plan.md: 30-day action plan w/ KPI targets
- docs/gbp/audit.{json,md}: raw capture of both branches

Key findings:
- MTPFUL2 has 5208 views/mo but 0 reviews — top priority
- Both branches: photos stale 1039-1579 days
- Name mismatch: GBP "Фулфилмент MTP Group" vs schema "MTP Group Fulfillment"
- Paused Google Ads campaign flagged

scripts/gbp-session/ gitignored (session cookies).

Co-Authored-By: claude-flow <ruv@ruv.net>
</commit_message>
<xml_diff>
--- a/docs/SEMANTIC_CORE_ROADMAP.xlsx
+++ b/docs/SEMANTIC_CORE_ROADMAP.xlsx
@@ -26,7 +26,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'🔄 v1 vs v2'!$A$1:$D$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'🏢 Competitors'!$A$1:$F$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'🔍 Top queries'!$A$1:$G$335</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'📅 Completion log'!$A$3:$F$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'📅 Completion log'!$A$3:$F$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -923,7 +923,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -976,12 +976,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Переписати home title + meta з ціною</t>
+          <t>GBP audit + optimization plan</t>
         </is>
       </c>
       <c r="C4" s="11" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>6058d76</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -1001,19 +1001,19 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>UA home вже мав 'від 18 грн' в title/desc. RU home extended LocalBusiness schema (logo, sameAs, priceRange, areaServed, knowsAbout) + WebSite schema. EN home title changed from '$0.40' to '€0.40/order</t>
+          <t>Built Playwright auth (scripts/gbp-auth.py) + audit (scripts/gbp-audit.py). Session stored in scripts/gbp-session/ (gitignored). Captured both branches, identified 5 priority actions: 1) reviews for M</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Organization schema для brand search</t>
+          <t>Claim Google Business Profile</t>
         </is>
       </c>
       <c r="C5" s="11" t="inlineStr">
@@ -1023,7 +1023,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6058d76</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>UA home had full LocalBusiness schema already. Extended RU + EN home with: logo, image, sameAs (FB/LinkedIn/Telegram), priceRange 'UAH 18 - UAH 650', aggregateRating, areaServed, knowsAbout. Fixed bro</t>
+          <t>Both branches already verified in group 'MTP Group фулфилмент' (id 111840383451580968640): MTPFUL1 (Щасливе) + MTPFUL2 (Білогородка). Audited via Playwright session. MTPFUL1: 4124 views/mo, 468 intera</t>
         </is>
       </c>
     </row>
@@ -1045,12 +1045,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Оновити /tsiny/ /tsenu/ /prices/ meta</t>
-        </is>
-      </c>
-      <c r="C6" s="13" t="inlineStr">
-        <is>
-          <t>✅ PARTIAL</t>
+          <t>Переписати home title + meta з ціною</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>✅ DONE</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>UA /tsiny/ and RU /tsenu/ already had '18 грн' in title/desc/FAQ schema — no change needed. EN /prices/ extended LocalBusiness schema with logo, sameAs, priceRange to match UA/RU quality.</t>
+          <t>UA home вже мав 'від 18 грн' в title/desc. RU home extended LocalBusiness schema (logo, sameAs, priceRange, areaServed, knowsAbout) + WebSite schema. EN home title changed from '$0.40' to '€0.40/order</t>
         </is>
       </c>
     </row>
@@ -1077,7 +1077,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Видалити дубль generate_lead/form_submit на EN thanks</t>
+          <t>Organization schema для brand search</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
@@ -1087,17 +1087,17 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>ff0bfe9</t>
+          <t>6058d76</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Phase 0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Fix A. en/thanks.astro: removed form_submit + generate_lead + dataLayer.push; kept only AdWords conversion event. Eliminates GA4 lead double-count for EN traffic.</t>
+          <t>UA home had full LocalBusiness schema already. Extended RU + EN home with: logo, image, sameAs (FB/LinkedIn/Telegram), priceRange 'UAH 18 - UAH 650', aggregateRating, areaServed, knowsAbout. Fixed bro</t>
         </is>
       </c>
     </row>
@@ -1109,27 +1109,27 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Видалити дубль GTM noscript iframe з 23 blog pages</t>
-        </is>
-      </c>
-      <c r="C8" s="11" t="inlineStr">
-        <is>
-          <t>✅ DONE</t>
+          <t>Оновити /tsiny/ /tsenu/ /prices/ meta</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>✅ PARTIAL</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>8a744c5</t>
+          <t>6058d76</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Phase 0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Fix B. Removed duplicate noscript iframe from 23 files; Base.astro:172 retained as single source of truth. 1 line deleted per file, no other changes.</t>
+          <t>UA /tsiny/ and RU /tsenu/ already had '18 грн' in title/desc/FAQ schema — no change needed. EN /prices/ extended LocalBusiness schema with logo, sameAs, priceRange to match UA/RU quality.</t>
         </is>
       </c>
     </row>
@@ -1141,7 +1141,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Tilda 301 clean sweep (59 legacy URLs)</t>
+          <t>Видалити дубль generate_lead/form_submit на EN thanks</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
@@ -1151,7 +1151,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>prior-session</t>
+          <t>ff0bfe9</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1161,7 +1161,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>vercel.json — 5 specific Tier 1 redirects + 3 catch-all patterns for /blog/tpost/, /ua/blog/tpost/, /en/blog/tpost/. All point directly to /ua/blog/ or /ua/about/ (no chained redirects). 132 redirects</t>
+          <t>Fix A. en/thanks.astro: removed form_submit + generate_lead + dataLayer.push; kept only AdWords conversion event. Eliminates GA4 lead double-count for EN traffic.</t>
         </is>
       </c>
     </row>
@@ -1173,54 +1173,96 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>Видалити дубль GTM noscript iframe з 23 blog pages</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>✅ DONE</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>8a744c5</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Fix B. Removed duplicate noscript iframe from 23 files; Base.astro:172 retained as single source of truth. 1 line deleted per file, no other changes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Tilda 301 clean sweep (59 legacy URLs)</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>✅ DONE</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>prior-session</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>vercel.json — 5 specific Tier 1 redirects + 3 catch-all patterns for /blog/tpost/, /ua/blog/tpost/, /en/blog/tpost/. All point directly to /ua/blog/ or /ua/about/ (no chained redirects). 132 redirects</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
           <t>GSC full audit + competitor research</t>
         </is>
       </c>
-      <c r="C10" s="11" t="inlineStr">
+      <c r="C12" s="11" t="inlineStr">
         <is>
           <t>✅ DONE</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>ff0bfe9</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>Analysis</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>Generated docs/gsc/full-pages.{csv,json}, full-queries.{csv,json}, opportunities.{csv,json}, competitor-gap-research.md. 178 pages, 334 queries, 29 clicks, 4329 impressions (90d baseline).</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Claim Google Business Profile</t>
-        </is>
-      </c>
-      <c r="C11" s="14" t="inlineStr">
-        <is>
-          <t>✅ MANUAL_USER_ACTION</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Phase 0</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>External task — user must claim at business.google.com. Recommended: entity name 'MTP Group Fulfillment', category 'Logistics service', both addresses (Щасливе + Білогородка), phone +380501444645, hou</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A3:F11"/>
+  <autoFilter ref="A3:F12"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
@@ -10938,9 +10980,9 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="F5" s="14" t="inlineStr">
-        <is>
-          <t>✅ MANUAL_USER_ACTION</t>
+      <c r="F5" s="15" t="inlineStr">
+        <is>
+          <t>✅ DONE</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -10948,9 +10990,19 @@
           <t>Brand CTR</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>External task — user must claim at business.google.com. Recommended: entity name 'MTP Group Fulfillment', category 'Logistics service', both addresses (Щасливе + Білогородка), phone +380501444645, hours Mo-Su 08:00-20:00.</t>
+          <t>Both branches already verified in group 'MTP Group фулфилмент' (id 111840383451580968640): MTPFUL1 (Щасливе) + MTPFUL2 (Білогородка). Audited via Playwright session. MTPFUL1: 4124 views/mo, 468 interactions. MTPFUL2: 5208 views/mo, 369 interactions, 0 reviews. Photos stale (1039 and 1579 days). Optimization plan in docs/gbp/optimization-plan.md.</t>
         </is>
       </c>
     </row>

</xml_diff>